<commit_message>
Update programme data and workflow animations
Update notes:

- Replace programme cluster metadata with years and regenerate programme import data.

- Keep database IDs aligned with alphabetical import order where safe.

- Add non-blocking inline loading panels between workflow stages.

- Animate priority ranking row movement and remove connector shimmer overlap.
</commit_message>
<xml_diff>
--- a/outputs/raw_data_cleaning/cleaned_raw_data_combined.xlsx
+++ b/outputs/raw_data_cleaning/cleaned_raw_data_combined.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="1" r:id="Rbc566847ba6b4980"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff" sheetId="2" r:id="R6ecdad78b7ad4036"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modules" sheetId="3" r:id="R64ba38575a0949c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programmes" sheetId="4" r:id="Re584f4e2d09841ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Common Modules" sheetId="5" r:id="Re2e29e84f45a4733"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Common Module Map" sheetId="6" r:id="Red410997f5b54a2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Rows" sheetId="7" r:id="Rdab94ed7111a4053"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleanup Notes" sheetId="8" r:id="R5d6cb2ba38224e89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="1" r:id="Rbf3e0eed4b004148"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staff" sheetId="2" r:id="R2566c9e93e9e49ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modules" sheetId="3" r:id="R954e1c1af3f146cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programmes" sheetId="4" r:id="Re64490349ba743e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Common Modules" sheetId="5" r:id="Ra43a181d39534e4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Common Module Map" sheetId="6" r:id="R84a0e07b402f402c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Rows" sheetId="7" r:id="Reeb13393d39045f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleanup Notes" sheetId="8" r:id="R400793ea3d5b428f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -186,12 +186,58 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="dk1"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="accent1"/>
-        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
+                <a:satMod val="110000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700">
@@ -41626,7 +41672,7 @@
   <x:cols>
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="33.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -41637,7 +41683,7 @@
         <x:v>name</x:v>
       </x:c>
       <x:c r="C1" s="4" t="str">
-        <x:v>cluster</x:v>
+        <x:v>years</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -41647,8 +41693,8 @@
       <x:c r="B2" s="9" t="str">
         <x:v>AAI</x:v>
       </x:c>
-      <x:c r="C2" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C2" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -41658,8 +41704,8 @@
       <x:c r="B3" s="9" t="str">
         <x:v>ACC</x:v>
       </x:c>
-      <x:c r="C3" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C3" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -41669,8 +41715,8 @@
       <x:c r="B4" s="9" t="str">
         <x:v>ASE</x:v>
       </x:c>
-      <x:c r="C4" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C4" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -41680,8 +41726,8 @@
       <x:c r="B5" s="9" t="str">
         <x:v>ATM</x:v>
       </x:c>
-      <x:c r="C5" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C5" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -41691,8 +41737,8 @@
       <x:c r="B6" s="9" t="str">
         <x:v>BAC</x:v>
       </x:c>
-      <x:c r="C6" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C6" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -41702,9 +41748,7 @@
       <x:c r="B7" s="9" t="str">
         <x:v>BCD</x:v>
       </x:c>
-      <x:c r="C7" s="9" t="str">
-        <x:v>Module host key</x:v>
-      </x:c>
+      <x:c r="C7" s="9"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="9" t="str">
@@ -41713,8 +41757,8 @@
       <x:c r="B8" s="9" t="str">
         <x:v>BICT</x:v>
       </x:c>
-      <x:c r="C8" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C8" s="9" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -41724,9 +41768,7 @@
       <x:c r="B9" s="9" t="str">
         <x:v>CBE</x:v>
       </x:c>
-      <x:c r="C9" s="9" t="str">
-        <x:v>Common Modules</x:v>
-      </x:c>
+      <x:c r="C9" s="9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="9" t="str">
@@ -41735,8 +41777,8 @@
       <x:c r="B10" s="9" t="str">
         <x:v>CDM</x:v>
       </x:c>
-      <x:c r="C10" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C10" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -41746,8 +41788,8 @@
       <x:c r="B11" s="9" t="str">
         <x:v>CEG</x:v>
       </x:c>
-      <x:c r="C11" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C11" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -41757,9 +41799,7 @@
       <x:c r="B12" s="9" t="str">
         <x:v>CLASIC</x:v>
       </x:c>
-      <x:c r="C12" s="9" t="str">
-        <x:v>Module host key</x:v>
-      </x:c>
+      <x:c r="C12" s="9"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="9" t="str">
@@ -41768,9 +41808,7 @@
       <x:c r="B13" s="9" t="str">
         <x:v>CPC</x:v>
       </x:c>
-      <x:c r="C13" s="9" t="str">
-        <x:v>Module host key</x:v>
-      </x:c>
+      <x:c r="C13" s="9"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="9" t="str">
@@ -41779,8 +41817,8 @@
       <x:c r="B14" s="9" t="str">
         <x:v>CVE</x:v>
       </x:c>
-      <x:c r="C14" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C14" s="9" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -41790,8 +41828,8 @@
       <x:c r="B15" s="9" t="str">
         <x:v>DSC</x:v>
       </x:c>
-      <x:c r="C15" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C15" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -41801,8 +41839,8 @@
       <x:c r="B16" s="9" t="str">
         <x:v>EDE</x:v>
       </x:c>
-      <x:c r="C16" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C16" s="9" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -41812,8 +41850,8 @@
       <x:c r="B17" s="9" t="str">
         <x:v>EEE</x:v>
       </x:c>
-      <x:c r="C17" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C17" s="9" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -41823,9 +41861,7 @@
       <x:c r="B18" s="9" t="str">
         <x:v>ENG</x:v>
       </x:c>
-      <x:c r="C18" s="9" t="str">
-        <x:v>Module host key</x:v>
-      </x:c>
+      <x:c r="C18" s="9"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="9" t="str">
@@ -41834,8 +41870,8 @@
       <x:c r="B19" s="9" t="str">
         <x:v>EPE</x:v>
       </x:c>
-      <x:c r="C19" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C19" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -41845,8 +41881,8 @@
       <x:c r="B20" s="9" t="str">
         <x:v>ESE</x:v>
       </x:c>
-      <x:c r="C20" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C20" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -41856,9 +41892,7 @@
       <x:c r="B21" s="9" t="str">
         <x:v>FCB</x:v>
       </x:c>
-      <x:c r="C21" s="9" t="str">
-        <x:v>Module host key</x:v>
-      </x:c>
+      <x:c r="C21" s="9"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="9" t="str">
@@ -41867,8 +41901,8 @@
       <x:c r="B22" s="9" t="str">
         <x:v>FDT</x:v>
       </x:c>
-      <x:c r="C22" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C22" s="9" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -41878,9 +41912,7 @@
       <x:c r="B23" s="9" t="str">
         <x:v>HSS</x:v>
       </x:c>
-      <x:c r="C23" s="9" t="str">
-        <x:v>Module host key</x:v>
-      </x:c>
+      <x:c r="C23" s="9"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="9" t="str">
@@ -41889,8 +41921,8 @@
       <x:c r="B24" s="9" t="str">
         <x:v>HTM</x:v>
       </x:c>
-      <x:c r="C24" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C24" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -41900,8 +41932,8 @@
       <x:c r="B25" s="9" t="str">
         <x:v>ICT</x:v>
       </x:c>
-      <x:c r="C25" s="9" t="str">
-        <x:v>Common Modules, Module host key</x:v>
+      <x:c r="C25" s="9" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -41911,9 +41943,7 @@
       <x:c r="B26" s="9" t="str">
         <x:v>IS</x:v>
       </x:c>
-      <x:c r="C26" s="9" t="str">
-        <x:v>Common Modules</x:v>
-      </x:c>
+      <x:c r="C26" s="9"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="9" t="str">
@@ -41922,8 +41952,8 @@
       <x:c r="B27" s="9" t="str">
         <x:v>MDME</x:v>
       </x:c>
-      <x:c r="C27" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C27" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -41933,8 +41963,8 @@
       <x:c r="B28" s="9" t="str">
         <x:v>MEC</x:v>
       </x:c>
-      <x:c r="C28" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C28" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -41944,8 +41974,8 @@
       <x:c r="B29" s="9" t="str">
         <x:v>METS</x:v>
       </x:c>
-      <x:c r="C29" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C29" s="9" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -41955,8 +41985,8 @@
       <x:c r="B30" s="9" t="str">
         <x:v>NAME</x:v>
       </x:c>
-      <x:c r="C30" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C30" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -41966,8 +41996,8 @@
       <x:c r="B31" s="9" t="str">
         <x:v>NUR</x:v>
       </x:c>
-      <x:c r="C31" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C31" s="9" t="n">
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -41977,9 +42007,7 @@
       <x:c r="B32" s="9" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="C32" s="9" t="str">
-        <x:v>Common Modules</x:v>
-      </x:c>
+      <x:c r="C32" s="9"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="9" t="str">
@@ -41988,9 +42016,7 @@
       <x:c r="B33" s="9" t="str">
         <x:v>PRE</x:v>
       </x:c>
-      <x:c r="C33" s="9" t="str">
-        <x:v>Common Modules</x:v>
-      </x:c>
+      <x:c r="C33" s="9"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="9" t="str">
@@ -41999,8 +42025,8 @@
       <x:c r="B34" s="9" t="str">
         <x:v>RSE</x:v>
       </x:c>
-      <x:c r="C34" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C34" s="9" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -42010,8 +42036,8 @@
       <x:c r="B35" s="9" t="str">
         <x:v>RTY</x:v>
       </x:c>
-      <x:c r="C35" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C35" s="9" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -42021,8 +42047,8 @@
       <x:c r="B36" s="9" t="str">
         <x:v>SBE</x:v>
       </x:c>
-      <x:c r="C36" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C36" s="9" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -42032,9 +42058,7 @@
       <x:c r="B37" s="9" t="str">
         <x:v>SE</x:v>
       </x:c>
-      <x:c r="C37" s="9" t="str">
-        <x:v>Common Modules</x:v>
-      </x:c>
+      <x:c r="C37" s="9"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="9" t="str">
@@ -42043,8 +42067,8 @@
       <x:c r="B38" s="9" t="str">
         <x:v>SLT</x:v>
       </x:c>
-      <x:c r="C38" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C38" s="9" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -42054,8 +42078,8 @@
       <x:c r="B39" s="9" t="str">
         <x:v>TCE</x:v>
       </x:c>
-      <x:c r="C39" s="9" t="str">
-        <x:v>Common Modules</x:v>
+      <x:c r="C39" s="9" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -42065,9 +42089,7 @@
       <x:c r="B40" s="9" t="str">
         <x:v>TITO</x:v>
       </x:c>
-      <x:c r="C40" s="9" t="str">
-        <x:v>Common Modules</x:v>
-      </x:c>
+      <x:c r="C40" s="9"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>